<commit_message>
🔄 MAJ automatique BRVM via GitHub Actions
</commit_message>
<xml_diff>
--- a/data/recommandations.xlsx
+++ b/data/recommandations.xlsx
@@ -476,10 +476,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>1414.26</v>
+        <v>1132.08</v>
       </c>
       <c r="E2" t="n">
         <v>281.89</v>
@@ -505,10 +505,10 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>1356.72</v>
+        <v>1089.89</v>
       </c>
       <c r="E3" t="n">
         <v>275.44</v>
@@ -534,10 +534,10 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>998.8</v>
+        <v>814.17</v>
       </c>
       <c r="E4" t="n">
         <v>212.11</v>
@@ -563,10 +563,10 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>965.45</v>
+        <v>777.09</v>
       </c>
       <c r="E5" t="n">
         <v>198.33</v>
@@ -592,10 +592,10 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>830.6</v>
+        <v>667.1</v>
       </c>
       <c r="E6" t="n">
         <v>169.85</v>
@@ -621,10 +621,10 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>778.66</v>
+        <v>624</v>
       </c>
       <c r="E7" t="n">
         <v>159.42</v>
@@ -650,10 +650,10 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>759.74</v>
+        <v>609.24</v>
       </c>
       <c r="E8" t="n">
         <v>154.95</v>
@@ -679,10 +679,10 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>656.79</v>
+        <v>529.37</v>
       </c>
       <c r="E9" t="n">
         <v>138.94</v>
@@ -708,10 +708,10 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>615.66</v>
+        <v>496.24</v>
       </c>
       <c r="E10" t="n">
         <v>127.92</v>
@@ -737,10 +737,10 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>504.88</v>
+        <v>403.72</v>
       </c>
       <c r="E11" t="n">
         <v>103.05</v>
@@ -824,10 +824,10 @@
         <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>11.76</v>
+        <v>14.75</v>
       </c>
       <c r="E14" t="n">
         <v>7.4</v>
@@ -839,27 +839,27 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ECOBANK TRANS. INCORP. TG (ETIT)</t>
+          <t>EVIOSYS PACKAGING SIEM CI (SEMC)</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>10.41</v>
+        <v>14.74</v>
       </c>
       <c r="E15" t="n">
-        <v>-2.94</v>
+        <v>7.33</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -868,27 +868,27 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SUCRIVOIRE (SCRC)</t>
+          <t>SICABLE CI (CABC)</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>10.17</v>
+        <v>12.48</v>
       </c>
       <c r="E16" t="n">
-        <v>-2.51</v>
+        <v>7.39</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -933,20 +933,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EVIOSYS PACKAGING SIEM CI (SEMC)</t>
+          <t>NEI-CEDA CI (NEIC)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>7.44</v>
+        <v>6.92</v>
       </c>
       <c r="E18" t="n">
-        <v>7.33</v>
+        <v>6.92</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -955,14 +955,14 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NEI-CEDA CI (NEIC)</t>
+          <t>TOTALENERGIES MARKETING CI (TTLC)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -972,10 +972,10 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>6.92</v>
+        <v>6.75</v>
       </c>
       <c r="E19" t="n">
-        <v>6.92</v>
+        <v>6.75</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -991,20 +991,20 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TOTALENERGIES MARKETING CI (TTLC)</t>
+          <t>SOLIBRA CI (SLBC)</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>6.75</v>
+        <v>4.74</v>
       </c>
       <c r="E20" t="n">
-        <v>6.75</v>
+        <v>7.49</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1013,14 +1013,14 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>➖ Neutre</t>
+          <t>👀 À surveiller</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CORIS BANK INTERNATIONAL (CBIBF)</t>
+          <t>ECOBANK TRANS. INCORP. TG (ETIT)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1030,10 +1030,10 @@
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>5.95</v>
+        <v>3.51</v>
       </c>
       <c r="E21" t="n">
-        <v>-1.55</v>
+        <v>-2.94</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1049,20 +1049,20 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SICABLE CI (CABC)</t>
+          <t>ONATEL BF (ONTBF)</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>5.03</v>
+        <v>3.19</v>
       </c>
       <c r="E22" t="n">
-        <v>7.39</v>
+        <v>-3.11</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1078,20 +1078,20 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SOLIBRA CI (SLBC)</t>
+          <t>SUCRIVOIRE (SCRC)</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>4.74</v>
+        <v>2.83</v>
       </c>
       <c r="E23" t="n">
-        <v>7.49</v>
+        <v>-2.51</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SITAB CI (STBC)</t>
+          <t>SMB CI (SMBC)</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1117,10 +1117,10 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>3.39</v>
+        <v>0.3</v>
       </c>
       <c r="E24" t="n">
-        <v>-1.9</v>
+        <v>6.66</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1136,20 +1136,20 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ONATEL BF (ONTBF)</t>
+          <t>BANK OF AFRICA CI (BOAC)</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25" t="n">
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>3.19</v>
+        <v>-1.32</v>
       </c>
       <c r="E25" t="n">
-        <v>-3.11</v>
+        <v>-1.32</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1158,27 +1158,27 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SMB CI (SMBC)</t>
+          <t>CORIS BANK INTERNATIONAL (CBIBF)</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>0.3</v>
+        <v>-1.55</v>
       </c>
       <c r="E26" t="n">
-        <v>6.66</v>
+        <v>-1.55</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1187,14 +1187,14 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BANK OF AFRICA CI (BOAC)</t>
+          <t>SITAB CI (STBC)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1204,10 +1204,10 @@
         <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>-1.32</v>
+        <v>-1.9</v>
       </c>
       <c r="E27" t="n">
-        <v>-1.32</v>
+        <v>-1.9</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1223,20 +1223,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>UNIWAX CI (UNXC)</t>
+          <t>BERNABE CI (BNBC)</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>-2.55</v>
+        <v>-2.24</v>
       </c>
       <c r="E28" t="n">
-        <v>-2.55</v>
+        <v>-1.58</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SOCIETE IVOIRIENNE DE BANQUE  (SIBC)</t>
+          <t>UNIWAX CI (UNXC)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1262,10 +1262,10 @@
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>-4.1</v>
+        <v>-2.55</v>
       </c>
       <c r="E29" t="n">
-        <v>-4.1</v>
+        <v>-2.55</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1281,49 +1281,49 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BERNABE CI (BNBC)</t>
+          <t>SOCIETE IVOIRIENNE DE BANQUE  (SIBC)</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>0</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>-6.37</v>
+        <v>-4.1</v>
       </c>
       <c r="E30" t="n">
-        <v>-1.58</v>
+        <v>-4.1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>🔴 Vente</t>
+          <t>🟡 Observer</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>⚠️ Risque de décrochage</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>UNILEVER CI (UNLC)</t>
+          <t>ECOBANK COTE D''IVOIRE (ECOC)</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>-6.4</v>
+        <v>-4.41</v>
       </c>
       <c r="E31" t="n">
-        <v>-6.86</v>
+        <v>-4.41</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ECOBANK COTE D''IVOIRE (ECOC)</t>
+          <t>UNILEVER CI (UNLC)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1378,10 +1378,10 @@
         <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>-9.74</v>
+        <v>-13.28</v>
       </c>
       <c r="E33" t="n">
-        <v>-4.41</v>
+        <v>-6.86</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1456,7 +1456,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>82151.91</v>
+        <v>21421.77</v>
       </c>
     </row>
     <row r="3">
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>70502.11</v>
+        <v>19146.55</v>
       </c>
     </row>
     <row r="4">
@@ -1476,7 +1476,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>24036.64</v>
+        <v>8380.01</v>
       </c>
     </row>
     <row r="5">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21519.53</v>
+        <v>7397.41</v>
       </c>
     </row>
     <row r="6">
@@ -1496,7 +1496,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13244.9</v>
+        <v>4964.48</v>
       </c>
     </row>
     <row r="7">
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10836.2</v>
+        <v>4194.43</v>
       </c>
     </row>
     <row r="8">
@@ -1516,7 +1516,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10051.1</v>
+        <v>3952.33</v>
       </c>
     </row>
     <row r="9">
@@ -1526,7 +1526,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6521.43</v>
+        <v>2811.54</v>
       </c>
     </row>
     <row r="10">
@@ -1536,7 +1536,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5428.85</v>
+        <v>2419.76</v>
       </c>
     </row>
     <row r="11">
@@ -1546,7 +1546,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3178.46</v>
+        <v>1529.78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>